<commit_message>
CGC Updates and Visualisations
</commit_message>
<xml_diff>
--- a/data/parameters_config/project_parameters.xlsx
+++ b/data/parameters_config/project_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rhartwell/PycharmProjects/VITRIFY/data/parameters_config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D359814-5DE9-3F42-9088-123D57C3BEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E255E7A-1012-2440-BEFD-EF8E33BDE3F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="122">
   <si>
     <t>Category</t>
   </si>
@@ -131,9 +131,6 @@
     <t>MAX_TRUCK_LOAD_KG</t>
   </si>
   <si>
-    <t>BREAKING_KGCO2_PER_M2</t>
-  </si>
-  <si>
     <t>DISASSEMBLY_KGCO2_PER_M2</t>
   </si>
   <si>
@@ -257,15 +254,6 @@
     <t>Density of sealant (kg/m3)</t>
   </si>
   <si>
-    <t>Linear mass of spacer (kg/m)</t>
-  </si>
-  <si>
-    <t>Embodied Carbon: 100% Recycled Glass (kgCO2e/kg)</t>
-  </si>
-  <si>
-    <t>Embodied Carbon: Virgin Float Glass (kgCO2e/kg)</t>
-  </si>
-  <si>
     <t>Embodied Carbon: PVB Interlayer (kgCO2e/kg)</t>
   </si>
   <si>
@@ -275,9 +263,6 @@
     <t>Emissions for disassembly process per m2</t>
   </si>
   <si>
-    <t>Site energy emissions per m2</t>
-  </si>
-  <si>
     <t>Energy emission for IGU assembly per m2</t>
   </si>
   <si>
@@ -348,6 +333,72 @@
   </si>
   <si>
     <t>Parameter for logic calculation (kgCO2/cavity Argon fill)</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>Parameter for logic calculation - implemented when undefined by user</t>
+  </si>
+  <si>
+    <t>Assumption based on average of poly-isobutylene, polysulfide</t>
+  </si>
+  <si>
+    <t>Linear mass of Aluminium spacer (kg/m) - material-based masses are converted based on user-input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EPD: EPD-IES-13054:001 </t>
+  </si>
+  <si>
+    <t>EPD-IES-0025026 Everlam PVB</t>
+  </si>
+  <si>
+    <t>EPD-IES-0011837:001</t>
+  </si>
+  <si>
+    <t>Embodied Carbon: Swiss Spacer (kgCO2e/linearmetre)</t>
+  </si>
+  <si>
+    <t>Embodied Carbon: Stainless Steel Spacer (kgCO2e/linearmetre)</t>
+  </si>
+  <si>
+    <t>Embodied Carbon: A1-A3 for 100% Recycled Glass (kgCO2e/kg)</t>
+  </si>
+  <si>
+    <t>Embodied Carbon: A1-A3 for Virgin Float Glass (kgCO2e/kg)</t>
+  </si>
+  <si>
+    <t>Defra 2024 Default value. Can be changed by user</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1007/s40940-022-00195-9</t>
+  </si>
+  <si>
+    <t>Parameter for logic calculation - not yet used</t>
+  </si>
+  <si>
+    <t>Saint Gobain Data - Magnetron coating</t>
+  </si>
+  <si>
+    <t>Saint Gobain Data - Tempering process</t>
+  </si>
+  <si>
+    <t>Saint Gobain Data - IGU manufacture</t>
+  </si>
+  <si>
+    <t>Emissions associated with deconstruction / disassembly of IGU from construction site [per m2]</t>
+  </si>
+  <si>
+    <t>Emissions associated with installation of IGU at construction site [per m2]</t>
+  </si>
+  <si>
+    <t>Based on assumption of 1.5 kg CO2/m2 GIA, and FSA:GIA = 0.3</t>
+  </si>
+  <si>
+    <t>BREAKING_KGCO2_PER_KG</t>
+  </si>
+  <si>
+    <t>Argon gas filling (0.016 m3 @ 1.699 kg/m3 Argon)</t>
   </si>
 </sst>
 </file>
@@ -371,15 +422,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -402,16 +465,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -716,14 +796,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="55.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -736,8 +817,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -748,10 +832,10 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -762,10 +846,10 @@
         <v>2500</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -776,10 +860,10 @@
         <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -790,10 +874,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -804,10 +888,10 @@
         <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -815,13 +899,16 @@
         <v>19</v>
       </c>
       <c r="C7">
-        <v>1400</v>
+        <v>1275</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+      <c r="E7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -829,13 +916,13 @@
         <v>20</v>
       </c>
       <c r="C8">
-        <v>6.4799999999999996E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -846,10 +933,13 @@
         <v>0.77</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+      <c r="E9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -860,10 +950,13 @@
         <v>1.29</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+      <c r="E10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -874,10 +967,13 @@
         <v>4.6829999999999998</v>
       </c>
       <c r="D11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+      <c r="E11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -888,10 +984,13 @@
         <v>3.51</v>
       </c>
       <c r="D12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+      <c r="E12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -902,10 +1001,10 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -916,10 +1015,10 @@
         <v>0.17</v>
       </c>
       <c r="D14" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -930,52 +1029,62 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="D15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+      <c r="E15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>6</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C16">
-        <v>0.27</v>
+        <v>0.91</v>
       </c>
       <c r="D16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+      <c r="E16" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>6</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C17">
         <v>0.3</v>
       </c>
       <c r="D17" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>6</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C18">
-        <v>0.39</v>
+        <f>0.47/2.5</f>
+        <v>0.188</v>
       </c>
       <c r="D18" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+      <c r="E18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -986,568 +1095,590 @@
         <v>24000</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>7</v>
       </c>
-      <c r="B20" t="s">
-        <v>32</v>
+      <c r="B20" s="6" t="s">
+        <v>120</v>
       </c>
       <c r="C20">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>7</v>
       </c>
-      <c r="B21" t="s">
-        <v>33</v>
+      <c r="B21" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>0.03</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C22">
-        <v>0.15</v>
+        <v>14.25</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+      <c r="E22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23">
-        <v>0.15</v>
+        <v>14.25</v>
       </c>
       <c r="D23" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="E23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+      <c r="E24" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>7</v>
       </c>
-      <c r="B25" t="s">
-        <v>37</v>
+      <c r="B25" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="C25">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>7</v>
       </c>
-      <c r="B26" t="s">
-        <v>38</v>
+      <c r="B26" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>7</v>
       </c>
-      <c r="B27" t="s">
-        <v>39</v>
+      <c r="B27" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="C27" s="2">
         <f>0.596*0.03</f>
         <v>1.788E-2</v>
       </c>
       <c r="D27" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+      <c r="E27" t="s">
+        <v>121</v>
+      </c>
+      <c r="F27">
+        <f>0.016*1.69</f>
+        <v>2.7039999999999998E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>7</v>
       </c>
-      <c r="B28" t="s">
-        <v>40</v>
+      <c r="B28" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D28" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>7</v>
       </c>
-      <c r="B29" t="s">
-        <v>41</v>
+      <c r="B29" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="C29">
-        <v>0.5</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="D29" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>7</v>
       </c>
-      <c r="B30" t="s">
-        <v>42</v>
+      <c r="B30" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="C30">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="D30" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>8</v>
       </c>
-      <c r="B31" t="s">
-        <v>43</v>
+      <c r="B31" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="C31">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D31" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32">
         <v>0.02</v>
       </c>
       <c r="D32" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>8</v>
       </c>
       <c r="B34" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C34">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D34" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C35">
         <v>0.2</v>
       </c>
       <c r="D35" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C36">
         <v>0.1</v>
       </c>
       <c r="D36" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C37">
         <v>0.2</v>
       </c>
       <c r="D37" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C38">
         <v>0.1</v>
       </c>
       <c r="D38" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C39">
         <v>0.1</v>
       </c>
       <c r="D39" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>9</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40">
         <v>0.8</v>
       </c>
       <c r="D40" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>9</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41">
         <v>0.4</v>
       </c>
       <c r="D41" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C42">
         <v>0.4</v>
       </c>
       <c r="D42" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>9</v>
       </c>
       <c r="B43" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C43">
         <v>0.52</v>
       </c>
       <c r="D43" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+      <c r="E43" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C44">
         <v>10</v>
       </c>
       <c r="D44" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C45">
         <v>0</v>
       </c>
       <c r="D45" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C46">
         <v>1000</v>
       </c>
       <c r="D46" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>10</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C47">
         <v>150</v>
       </c>
       <c r="D47" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C48">
         <v>80</v>
       </c>
       <c r="D48" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D49" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>12</v>
       </c>
       <c r="B50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C50">
         <v>1.6</v>
       </c>
       <c r="D50" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>12</v>
       </c>
       <c r="B51" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51">
         <v>50</v>
       </c>
       <c r="D51" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C52">
         <v>50</v>
       </c>
       <c r="D52" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C53">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="D53" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C54">
-        <v>6.2E-2</v>
+        <v>7.2400000000000006E-2</v>
       </c>
       <c r="D54" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+      <c r="E54" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C55">
         <v>500</v>
       </c>
       <c r="D55" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C56" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D56" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C57" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D57" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C58">
         <v>24</v>
       </c>
       <c r="D58" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>13</v>
       </c>
       <c r="B59" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C59">
         <v>25</v>
       </c>
       <c r="D59" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>